<commit_message>
Update Schedule.xlsx after scheduled run
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Emails" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -798,6 +798,11 @@
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sent (04/09/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="inlineStr">
@@ -816,6 +821,11 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>&lt;p&gt;Hello,&lt;/p&gt;&lt;p&gt;This is a demo test email sent via the GitHub Actions workflow to confirm the mass mail scheduler is working end-to-end.&lt;/p&gt;&lt;p&gt;Regards,&lt;br&gt;Mass Mail Scheduler&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sent (04/09/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add trial cron times and CC/new schedule rows; fill missing Date
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="165" formatCode="[$-409]dd/mmm/yy;@"/>
     <numFmt numFmtId="166" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,6 +85,11 @@
       <family val="2"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -130,7 +135,7 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -168,6 +173,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -781,6 +789,11 @@
           <t>legal@indigopaints.com</t>
         </is>
       </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>indigoschemes@indigopaints.com</t>
+        </is>
+      </c>
       <c r="G2" s="8" t="n">
         <v>46269</v>
       </c>
@@ -792,7 +805,7 @@
       <c r="I2" s="15" t="inlineStr">
         <is>
           <t>&lt;p&gt;Dear Team,&lt;/p&gt;
-&lt;p&gt;Employer professional tax due date &lt;/p&gt;
+&lt;p&gt;Employer professional tax due date 04-09-2026 &lt;/p&gt;
 &lt;p&gt;Regards,&lt;br&gt;
 Yuvraj Musale&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
@@ -805,8 +818,13 @@
           <t>indigoschemes@indigopaints.com</t>
         </is>
       </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>indigoschemes@indigopaints.com</t>
+        </is>
+      </c>
       <c r="G3" s="8" t="n">
-        <v>46274</v>
+        <v>46269</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -820,12 +838,62 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="4" t="n"/>
-      <c r="G4" s="8" t="n"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="5" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>legal@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>indigoschemes@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>ESIC</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;ESIC due date &lt;/p&gt;
+&lt;p&gt;Regards,&lt;br&gt;
+Youraj Musale&lt;br&gt;
+Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="116" customHeight="1">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>legal@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>indigoschemes@indigopaints.com</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Employee professional tax due date </t>
+        </is>
+      </c>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dear Team,&lt;/p&gt;
+&lt;p&gt;Employee professional tax due date 04-09-2026 &lt;/p&gt;
+&lt;p&gt;Regards,&lt;br&gt;
+Youraj Musale&lt;br&gt;
+Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="5" t="n"/>
@@ -1063,6 +1131,8 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge sent-status updates from GitHub into local Schedule.xlsx
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -811,6 +811,11 @@
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sent (04/09/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" s="4" t="inlineStr">
@@ -834,6 +839,11 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>&lt;p&gt;Hello,&lt;/p&gt;&lt;p&gt;This is a demo test email sent via the GitHub Actions workflow to confirm the mass mail scheduler is working end-to-end.&lt;/p&gt;&lt;p&gt;Regards,&lt;br&gt;Mass Mail Scheduler&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Sent (04/09/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adopt sent statuses from latest scheduled run
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Schedule.xlsx
+++ b/Schedule.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emails" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Emails" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -875,6 +875,11 @@
 Indigo Paints Ltd.&lt;/p&gt;</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Sent (04/09/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="116" customHeight="1">
       <c r="B5" s="5" t="inlineStr">
@@ -902,6 +907,11 @@
 &lt;p&gt;Regards,&lt;br&gt;
 Youraj Musale&lt;br&gt;
 Indigo Paints Ltd.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Sent (04/09/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>